<commit_message>
Corrida | ARG-PIB | 2026-09-22 10:08:00.784686
</commit_message>
<xml_diff>
--- a/indicadores/ARG-PIB_out.xlsx
+++ b/indicadores/ARG-PIB_out.xlsx
@@ -110,13 +110,13 @@
     <t xml:space="preserve">Fecha</t>
   </si>
   <si>
-    <t xml:space="preserve">18/09/2026</t>
+    <t xml:space="preserve">22/09/2026</t>
   </si>
   <si>
     <t xml:space="preserve">Usuario</t>
   </si>
   <si>
-    <t xml:space="preserve">vcorvalan</t>
+    <t xml:space="preserve">pcohan</t>
   </si>
   <si>
     <t xml:space="preserve">fecha</t>

</xml_diff>

<commit_message>
Corrida | ARG-PIB | 2026-09-22 10:23:45.883885
</commit_message>
<xml_diff>
--- a/indicadores/ARG-PIB_out.xlsx
+++ b/indicadores/ARG-PIB_out.xlsx
@@ -1557,7 +1557,7 @@
       <c r="B11"/>
       <c r="C11"/>
       <c r="D11" t="n">
-        <v>0.721975929584775</v>
+        <v>0.721976070980911</v>
       </c>
       <c r="E11"/>
       <c r="F11"/>
@@ -1615,7 +1615,7 @@
       <c r="B15"/>
       <c r="C15"/>
       <c r="D15" t="n">
-        <v>0.5212492428998</v>
+        <v>0.521249447069034</v>
       </c>
       <c r="E15"/>
       <c r="F15"/>
@@ -1685,7 +1685,7 @@
       <c r="B20"/>
       <c r="C20"/>
       <c r="D20" t="n">
-        <v>0.153979925743781</v>
+        <v>0.155406451165819</v>
       </c>
       <c r="E20"/>
       <c r="F20"/>
@@ -1715,7 +1715,7 @@
       <c r="B22"/>
       <c r="C22"/>
       <c r="D22" t="n">
-        <v>0.000121431265441804</v>
+        <v>0.000122214878132112</v>
       </c>
       <c r="E22"/>
       <c r="F22"/>
@@ -15856,7 +15856,7 @@
         <v>318</v>
       </c>
       <c r="B5" s="1" t="n">
-        <v>-0.00927490880339486</v>
+        <v>-0.00927488978475926</v>
       </c>
     </row>
     <row r="6">
@@ -15864,7 +15864,7 @@
         <v>319</v>
       </c>
       <c r="B6" s="1" t="n">
-        <v>0.125728228285431</v>
+        <v>0.125727948774284</v>
       </c>
     </row>
     <row r="7">
@@ -15872,7 +15872,7 @@
         <v>320</v>
       </c>
       <c r="B7" s="1" t="n">
-        <v>0.372731563800158</v>
+        <v>0.372731159685304</v>
       </c>
     </row>
     <row r="8">
@@ -15880,7 +15880,7 @@
         <v>321</v>
       </c>
       <c r="B8" s="1" t="n">
-        <v>0.634641684549077</v>
+        <v>0.634641391983953</v>
       </c>
     </row>
     <row r="9">
@@ -15888,7 +15888,7 @@
         <v>322</v>
       </c>
       <c r="B9" s="1" t="n">
-        <v>0.721975929584775</v>
+        <v>0.721976070980911</v>
       </c>
     </row>
     <row r="10">
@@ -15896,7 +15896,7 @@
         <v>323</v>
       </c>
       <c r="B10" s="1" t="n">
-        <v>0.512483550579467</v>
+        <v>0.512484005675732</v>
       </c>
     </row>
     <row r="11">
@@ -15904,7 +15904,7 @@
         <v>324</v>
       </c>
       <c r="B11" s="1" t="n">
-        <v>0.162111729649501</v>
+        <v>0.162112305279211</v>
       </c>
     </row>
     <row r="12">
@@ -15912,7 +15912,7 @@
         <v>325</v>
       </c>
       <c r="B12" s="1" t="n">
-        <v>-0.0409973047744464</v>
+        <v>-0.040997019684774</v>
       </c>
     </row>
     <row r="13">
@@ -15920,7 +15920,7 @@
         <v>326</v>
       </c>
       <c r="B13" s="1" t="n">
-        <v>-0.0861678775623498</v>
+        <v>-0.0861678969513603</v>
       </c>
     </row>
     <row r="14">

</xml_diff>

<commit_message>
Corrida | ARG-PIB | 2026-10-13 15:02:50.06775
</commit_message>
<xml_diff>
--- a/indicadores/ARG-PIB_out.xlsx
+++ b/indicadores/ARG-PIB_out.xlsx
@@ -110,7 +110,7 @@
     <t xml:space="preserve">Fecha</t>
   </si>
   <si>
-    <t xml:space="preserve">22/09/2026</t>
+    <t xml:space="preserve">13/10/2026</t>
   </si>
   <si>
     <t xml:space="preserve">Usuario</t>
@@ -1557,7 +1557,7 @@
       <c r="B11"/>
       <c r="C11"/>
       <c r="D11" t="n">
-        <v>0.721976070980911</v>
+        <v>0.72279549133684</v>
       </c>
       <c r="E11"/>
       <c r="F11"/>
@@ -1615,7 +1615,7 @@
       <c r="B15"/>
       <c r="C15"/>
       <c r="D15" t="n">
-        <v>0.521249447069034</v>
+        <v>0.522433322296865</v>
       </c>
       <c r="E15"/>
       <c r="F15"/>
@@ -1685,7 +1685,7 @@
       <c r="B20"/>
       <c r="C20"/>
       <c r="D20" t="n">
-        <v>0.155406451165819</v>
+        <v>0.15189726240943</v>
       </c>
       <c r="E20"/>
       <c r="F20"/>
@@ -1715,7 +1715,7 @@
       <c r="B22"/>
       <c r="C22"/>
       <c r="D22" t="n">
-        <v>0.000122214878132112</v>
+        <v>0.000112763772148089</v>
       </c>
       <c r="E22"/>
       <c r="F22"/>
@@ -15856,7 +15856,7 @@
         <v>318</v>
       </c>
       <c r="B5" s="1" t="n">
-        <v>-0.00927488978475926</v>
+        <v>-0.00570770954043151</v>
       </c>
     </row>
     <row r="6">
@@ -15864,7 +15864,7 @@
         <v>319</v>
       </c>
       <c r="B6" s="1" t="n">
-        <v>0.125727948774284</v>
+        <v>0.125943585415831</v>
       </c>
     </row>
     <row r="7">
@@ -15872,7 +15872,7 @@
         <v>320</v>
       </c>
       <c r="B7" s="1" t="n">
-        <v>0.372731159685304</v>
+        <v>0.371203886025271</v>
       </c>
     </row>
     <row r="8">
@@ -15880,7 +15880,7 @@
         <v>321</v>
       </c>
       <c r="B8" s="1" t="n">
-        <v>0.634641391983953</v>
+        <v>0.63381822983202</v>
       </c>
     </row>
     <row r="9">
@@ -15888,7 +15888,7 @@
         <v>322</v>
       </c>
       <c r="B9" s="1" t="n">
-        <v>0.721976070980911</v>
+        <v>0.72279549133684</v>
       </c>
     </row>
     <row r="10">
@@ -15896,7 +15896,7 @@
         <v>323</v>
       </c>
       <c r="B10" s="1" t="n">
-        <v>0.512484005675732</v>
+        <v>0.513245435976576</v>
       </c>
     </row>
     <row r="11">
@@ -15904,7 +15904,7 @@
         <v>324</v>
       </c>
       <c r="B11" s="1" t="n">
-        <v>0.162112305279211</v>
+        <v>0.160244202673772</v>
       </c>
     </row>
     <row r="12">
@@ -15912,7 +15912,7 @@
         <v>325</v>
       </c>
       <c r="B12" s="1" t="n">
-        <v>-0.040997019684774</v>
+        <v>-0.0415902918702597</v>
       </c>
     </row>
     <row r="13">
@@ -15920,7 +15920,7 @@
         <v>326</v>
       </c>
       <c r="B13" s="1" t="n">
-        <v>-0.0861678969513603</v>
+        <v>-0.0886746811739005</v>
       </c>
     </row>
     <row r="14">

</xml_diff>